<commit_message>
Added all resources in main.py
</commit_message>
<xml_diff>
--- a/Data/tables/main_event_attribute_info.xlsx
+++ b/Data/tables/main_event_attribute_info.xlsx
@@ -431,19 +431,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>case</t>
+          <t>response_status_code</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>planned_operation_time</t>
+          <t>requested_service_url</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -455,31 +455,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>time:timestamp</t>
+          <t>identifier:id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>lifecycle:transition</t>
+          <t>parameters</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>dict</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>org:resource</t>
+          <t>SubProcessID</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -491,7 +491,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>case:concept:name</t>
+          <t>complete_service_time</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -503,19 +503,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>response_status_code</t>
+          <t>current_task</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>current_task</t>
+          <t>org:resource</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -527,19 +527,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>requested_service_url</t>
+          <t>human_workstation_green_button_pressed</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>process_model_id</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -551,19 +551,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>parameters</t>
+          <t>time:timestamp</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>dict</t>
+          <t>datetime</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>process_model_id</t>
+          <t>case</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SubProcessID</t>
+          <t>concept:name</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>concept:name</t>
+          <t>planned_operation_time</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>identifier:id</t>
+          <t>lifecycle:transition</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -611,7 +611,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lifecycle:state</t>
+          <t>case:concept:name</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -623,43 +623,43 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>operation_end_time</t>
+          <t>unsatisfied_condition_description</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>unsatisfied_condition_description</t>
+          <t>operation_end_time</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>datetime</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>human_workstation_green_button_pressed</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>complete_service_time</t>
+          <t>lifecycle:state</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">

</xml_diff>

<commit_message>
small changes + finnished anomaly detection pipeline
</commit_message>
<xml_diff>
--- a/Data/tables/main_event_attribute_info.xlsx
+++ b/Data/tables/main_event_attribute_info.xlsx
@@ -431,19 +431,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>response_status_code</t>
+          <t>process_model_id</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>requested_service_url</t>
+          <t>lifecycle:state</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -455,31 +455,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>identifier:id</t>
+          <t>time:timestamp</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>datetime</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>parameters</t>
+          <t>human_workstation_green_button_pressed</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>dict</t>
+          <t>float</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SubProcessID</t>
+          <t>org:resource</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -491,7 +491,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>complete_service_time</t>
+          <t>lifecycle:transition</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -503,19 +503,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>current_task</t>
+          <t>response_status_code</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>org:resource</t>
+          <t>case</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -527,43 +527,43 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>human_workstation_green_button_pressed</t>
+          <t>concept:name</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>process_model_id</t>
+          <t>operation_end_time</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>datetime</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>time:timestamp</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>case</t>
+          <t>case:concept:name</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>concept:name</t>
+          <t>complete_service_time</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>planned_operation_time</t>
+          <t>unsatisfied_condition_description</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lifecycle:transition</t>
+          <t>planned_operation_time</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -611,7 +611,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>case:concept:name</t>
+          <t>SubProcessID</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>unsatisfied_condition_description</t>
+          <t>current_task</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -635,19 +635,19 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>operation_end_time</t>
+          <t>identifier:id</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>requested_service_url</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -659,12 +659,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lifecycle:state</t>
+          <t>parameters</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>dict</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
finnished, before val/test switch
</commit_message>
<xml_diff>
--- a/Data/tables/main_event_attribute_info.xlsx
+++ b/Data/tables/main_event_attribute_info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,7 +431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>process_model_id</t>
+          <t>org:resource</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -443,55 +443,55 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lifecycle:state</t>
+          <t>operation_end_time</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>datetime</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>time:timestamp</t>
+          <t>lifecycle:state</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>human_workstation_green_button_pressed</t>
+          <t>unsatisfied_condition_description</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>org:resource</t>
+          <t>time:timestamp</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>datetime</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>lifecycle:transition</t>
+          <t>case</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -503,19 +503,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>response_status_code</t>
+          <t>fier:id</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>case</t>
+          <t>SubProcessID</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>concept:name</t>
+          <t>current_task</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -539,19 +539,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>operation_end_time</t>
+          <t>human_workstation_green_button_pressed</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>float</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>requested_service_url</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>case:concept:name</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>complete_service_time</t>
+          <t>identifier:id</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -587,19 +587,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>unsatisfied_condition_description</t>
+          <t>parameters</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>dict</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>planned_operation_time</t>
+          <t>process_model_id</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -611,7 +611,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SubProcessID</t>
+          <t>lifecycle:transition</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>current_task</t>
+          <t>complete_service_time</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>identifier:id</t>
+          <t>concept:name</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>requested_service_url</t>
+          <t>planned_operation_time</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -659,12 +659,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>parameters</t>
+          <t>response_status_code</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>dict</t>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>case:concept:name</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>str</t>
         </is>
       </c>
     </row>

</xml_diff>